<commit_message>
version avec graphique chaque indicateur
</commit_message>
<xml_diff>
--- a/data/AGRICULTURE.xlsx
+++ b/data/AGRICULTURE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SekouDRAME\Desktop\ANSD_KAFFRINE\Dashboard_SRSD_Kaffrine\dashboard_multi_sectoriel_kaffrine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D659A06A-7652-4C1A-A82F-8C95C96B6811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027247A1-7458-4207-A339-6D68E9D3A7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -585,6 +585,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1028,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AC5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.35">
@@ -1117,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="AC6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.35">
@@ -1206,7 +1209,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.35">
@@ -1295,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1384,7 +1387,7 @@
         <v>4</v>
       </c>
       <c r="AC9">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1829,7 +1832,7 @@
         <v>4</v>
       </c>
       <c r="AC14">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1918,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="AC15">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -2007,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="AC16">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.35">
@@ -2096,7 +2099,7 @@
         <v>3</v>
       </c>
       <c r="AC17">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.35">
@@ -2185,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.35">
@@ -2630,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="AC23">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.35">
@@ -2719,7 +2722,7 @@
         <v>10</v>
       </c>
       <c r="AC24">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.35">
@@ -2808,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="AC25">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.35">
@@ -2897,7 +2900,7 @@
         <v>2</v>
       </c>
       <c r="AC26">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.35">
@@ -2986,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.35">
@@ -3342,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="AC31">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.35">
@@ -3431,7 +3434,7 @@
         <v>2</v>
       </c>
       <c r="AC32">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.35">
@@ -3520,7 +3523,7 @@
         <v>5</v>
       </c>
       <c r="AC33">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.35">
@@ -3609,7 +3612,7 @@
         <v>10</v>
       </c>
       <c r="AC34">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mise a jour année a 2025
</commit_message>
<xml_diff>
--- a/data/AGRICULTURE.xlsx
+++ b/data/AGRICULTURE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SekouDRAME\Desktop\ANSD_KAFFRINE\Dashboard_SRSD_Kaffrine\dashboard_multi_sectoriel_kaffrine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{027247A1-7458-4207-A339-6D68E9D3A7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238B2BF4-2447-45A1-B3CF-07B1C2C645D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1031,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AC5">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.35">
@@ -1120,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="AC6">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.35">
@@ -1209,7 +1209,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.35">
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1387,7 +1387,7 @@
         <v>4</v>
       </c>
       <c r="AC9">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1832,7 +1832,7 @@
         <v>4</v>
       </c>
       <c r="AC14">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="AC15">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -2010,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="AC16">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.35">
@@ -2099,7 +2099,7 @@
         <v>3</v>
       </c>
       <c r="AC17">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.35">
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="AC23">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.35">
@@ -2722,7 +2722,7 @@
         <v>10</v>
       </c>
       <c r="AC24">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.35">
@@ -2811,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="AC25">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.35">
@@ -2900,7 +2900,7 @@
         <v>2</v>
       </c>
       <c r="AC26">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.35">
@@ -2989,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.35">
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="AC31">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.35">
@@ -3434,7 +3434,7 @@
         <v>2</v>
       </c>
       <c r="AC32">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.35">
@@ -3523,7 +3523,7 @@
         <v>5</v>
       </c>
       <c r="AC33">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.35">
@@ -3612,7 +3612,7 @@
         <v>10</v>
       </c>
       <c r="AC34">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changement agriculture.xlsx et data)loader.py
</commit_message>
<xml_diff>
--- a/data/AGRICULTURE.xlsx
+++ b/data/AGRICULTURE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SekouDRAME\Desktop\ANSD_KAFFRINE\Dashboard_SRSD_Kaffrine\dashboard_multi_sectoriel_kaffrine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238B2BF4-2447-45A1-B3CF-07B1C2C645D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B87DA8CE-4196-4B5A-B2CB-A934494BF720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1031,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AC5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.35">
@@ -1120,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="AC6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.35">
@@ -1209,7 +1209,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.35">
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1387,7 +1387,7 @@
         <v>4</v>
       </c>
       <c r="AC9">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1832,7 +1832,7 @@
         <v>4</v>
       </c>
       <c r="AC14">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="AC15">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -2010,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="AC16">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.35">
@@ -2099,7 +2099,7 @@
         <v>3</v>
       </c>
       <c r="AC17">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.35">
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="AC23">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.35">
@@ -2722,7 +2722,7 @@
         <v>10</v>
       </c>
       <c r="AC24">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.35">
@@ -2811,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="AC25">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.35">
@@ -2900,7 +2900,7 @@
         <v>2</v>
       </c>
       <c r="AC26">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.35">
@@ -2989,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.35">
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="AC31">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.35">
@@ -3434,7 +3434,7 @@
         <v>2</v>
       </c>
       <c r="AC32">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.35">
@@ -3523,7 +3523,7 @@
         <v>5</v>
       </c>
       <c r="AC33">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.35">
@@ -3612,7 +3612,7 @@
         <v>10</v>
       </c>
       <c r="AC34">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update data_loader.py et agriculture.xlsx
</commit_message>
<xml_diff>
--- a/data/AGRICULTURE.xlsx
+++ b/data/AGRICULTURE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SekouDRAME\Desktop\ANSD_KAFFRINE\Dashboard_SRSD_Kaffrine\dashboard_multi_sectoriel_kaffrine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C669A9-52F0-4FFD-AAA9-59D1A27BF6E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE607A7A-B37B-4DE4-BA75-252A4A26843A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1031,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AC5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.35">
@@ -1120,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="AC6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.35">
@@ -1209,7 +1209,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.35">
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1387,7 +1387,7 @@
         <v>4</v>
       </c>
       <c r="AC9">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1832,7 +1832,7 @@
         <v>4</v>
       </c>
       <c r="AC14">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="AC15">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -2010,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="AC16">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.35">
@@ -2099,7 +2099,7 @@
         <v>3</v>
       </c>
       <c r="AC17">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.35">
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="AC23">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.35">
@@ -2722,7 +2722,7 @@
         <v>10</v>
       </c>
       <c r="AC24">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.35">
@@ -2811,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="AC25">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.35">
@@ -2900,7 +2900,7 @@
         <v>2</v>
       </c>
       <c r="AC26">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.35">
@@ -2989,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.35">
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="AC31">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.35">
@@ -3434,7 +3434,7 @@
         <v>2</v>
       </c>
       <c r="AC32">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.35">
@@ -3523,7 +3523,7 @@
         <v>5</v>
       </c>
       <c r="AC33">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.35">
@@ -3612,7 +3612,7 @@
         <v>10</v>
       </c>
       <c r="AC34">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remplace annee par 2025
</commit_message>
<xml_diff>
--- a/data/AGRICULTURE.xlsx
+++ b/data/AGRICULTURE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SekouDRAME\Desktop\ANSD_KAFFRINE\Dashboard_SRSD_Kaffrine\dashboard_multi_sectoriel_kaffrine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE607A7A-B37B-4DE4-BA75-252A4A26843A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E619FE6A-D6C9-4148-BFE1-49DA11564FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1031,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AC5">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.35">
@@ -1120,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="AC6">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.35">
@@ -1209,7 +1209,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.35">
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1387,7 +1387,7 @@
         <v>4</v>
       </c>
       <c r="AC9">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1832,7 +1832,7 @@
         <v>4</v>
       </c>
       <c r="AC14">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="AC15">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -2010,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="AC16">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.35">
@@ -2099,7 +2099,7 @@
         <v>3</v>
       </c>
       <c r="AC17">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.35">
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="AC23">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.35">
@@ -2722,7 +2722,7 @@
         <v>10</v>
       </c>
       <c r="AC24">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.35">
@@ -2811,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="AC25">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.35">
@@ -2900,7 +2900,7 @@
         <v>2</v>
       </c>
       <c r="AC26">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.35">
@@ -2989,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.35">
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="AC31">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.35">
@@ -3434,7 +3434,7 @@
         <v>2</v>
       </c>
       <c r="AC32">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.35">
@@ -3523,7 +3523,7 @@
         <v>5</v>
       </c>
       <c r="AC33">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.35">
@@ -3612,7 +3612,7 @@
         <v>10</v>
       </c>
       <c r="AC34">
-        <v>2026</v>
+        <v>2025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changement loader_data.py et agriculture.xlsx
</commit_message>
<xml_diff>
--- a/data/AGRICULTURE.xlsx
+++ b/data/AGRICULTURE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SekouDRAME\Desktop\ANSD_KAFFRINE\Dashboard_SRSD_Kaffrine\dashboard_multi_sectoriel_kaffrine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E619FE6A-D6C9-4148-BFE1-49DA11564FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44BEA64B-8069-4B1F-84DD-47B45C9EA73A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1031,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="AC5">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.35">
@@ -1120,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="AC6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.35">
@@ -1209,7 +1209,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.35">
@@ -1298,7 +1298,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.35">
@@ -1387,7 +1387,7 @@
         <v>4</v>
       </c>
       <c r="AC9">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="10" spans="1:29" x14ac:dyDescent="0.35">
@@ -1832,7 +1832,7 @@
         <v>4</v>
       </c>
       <c r="AC14">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.35">
@@ -1921,7 +1921,7 @@
         <v>4</v>
       </c>
       <c r="AC15">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.35">
@@ -2010,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="AC16">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="17" spans="1:29" x14ac:dyDescent="0.35">
@@ -2099,7 +2099,7 @@
         <v>3</v>
       </c>
       <c r="AC17">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="18" spans="1:29" x14ac:dyDescent="0.35">
@@ -2188,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="19" spans="1:29" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="AC23">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.35">
@@ -2722,7 +2722,7 @@
         <v>10</v>
       </c>
       <c r="AC24">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.35">
@@ -2811,7 +2811,7 @@
         <v>7</v>
       </c>
       <c r="AC25">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.35">
@@ -2900,7 +2900,7 @@
         <v>2</v>
       </c>
       <c r="AC26">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.35">
@@ -2989,7 +2989,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.35">
@@ -3345,7 +3345,7 @@
         <v>1</v>
       </c>
       <c r="AC31">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.35">
@@ -3434,7 +3434,7 @@
         <v>2</v>
       </c>
       <c r="AC32">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.35">
@@ -3523,7 +3523,7 @@
         <v>5</v>
       </c>
       <c r="AC33">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.35">
@@ -3612,7 +3612,7 @@
         <v>10</v>
       </c>
       <c r="AC34">
-        <v>2025</v>
+        <v>2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>